<commit_message>
Update project docs, bibliography, and evidence README
Add Office temp-file pattern (~$*) to .gitignore. Replace/refresh multiple deliverables and registry files (docx, pdf, xlsx) under documentos/, entregas/ and gestion/registros/ with updated versions. Revise evidencias/semana-01/README.md: rename section to "Identificación y evidencia independiente", update the members table with roles/placeholders and a note about pending confirmations, and mark initial checklist items as completed. Expand and correct fuentes/semana-01/bibliografia.md: fix Gao et al. author list and citation, and add several regulatory and data-protection references (MVCS, SST laws, ANPD, etc.).
</commit_message>
<xml_diff>
--- a/entregas/semana-01/TISG_E01_S01_RegistrosRadar_2026-09-04.xlsx
+++ b/entregas/semana-01/TISG_E01_S01_RegistrosRadar_2026-09-04.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\TISG_ProyectoIntegrador_Grupo1_2026-2\gestion\registros\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D4621C4C-CC06-4D0F-8846-CF71085B7615}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1362F59F-0C56-4798-8943-FE68A2B9DBF5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="300" uniqueCount="223">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="332" uniqueCount="250">
   <si>
     <t>ID</t>
   </si>
@@ -542,9 +542,6 @@
     <t>F-12</t>
   </si>
   <si>
-    <t>Gao et al. - AI in Construction Project Management: systematic review</t>
-  </si>
-  <si>
     <t>IA aplicada a costos, tiempo y seguridad; límites de generalización y datos.</t>
   </si>
   <si>
@@ -665,27 +662,15 @@
     <t>Anthony Romani</t>
   </si>
   <si>
-    <t>Sustituir Anthony Romani por el nombre real antes de entregar.</t>
-  </si>
-  <si>
     <t>Max Astuhuaman</t>
   </si>
   <si>
-    <t>Sustituir Max Astuhuaman por el nombre real antes de entregar.</t>
-  </si>
-  <si>
     <t>Guillermo Calle</t>
   </si>
   <si>
-    <t>Sustituir Guillermo Calle por el nombre real antes de entregar.</t>
-  </si>
-  <si>
     <t>Pablo</t>
   </si>
   <si>
-    <t>Sustituir Pablo por el nombre real antes de entregar.</t>
-  </si>
-  <si>
     <t>Documento: secciones 2, 3 y 8</t>
   </si>
   <si>
@@ -693,6 +678,102 @@
   </si>
   <si>
     <t>Documento: secciones 4 y 7; revisión integral</t>
+  </si>
+  <si>
+    <t>Nombre real registrado.</t>
+  </si>
+  <si>
+    <t>Fuente / evidencia</t>
+  </si>
+  <si>
+    <t>Definición académica del caso y criterio de anonimización del repositorio.</t>
+  </si>
+  <si>
+    <t>Levantamiento funcional anonimizado; sección 3 del documento.</t>
+  </si>
+  <si>
+    <t>Levantamiento funcional anonimizado; sección 3.1 del documento.</t>
+  </si>
+  <si>
+    <t>Levantamiento funcional anonimizado; flujo AS-IS de la sección 3.</t>
+  </si>
+  <si>
+    <t>Levantamiento funcional anonimizado; integración pendiente de validación.</t>
+  </si>
+  <si>
+    <t>Levantamiento funcional anonimizado; brecha de la sección 3.3.</t>
+  </si>
+  <si>
+    <t>Sin evidencia independiente; requiere entrevista o validación del equipo TI.</t>
+  </si>
+  <si>
+    <t>Criterio de confidencialidad y protección de datos del repositorio.</t>
+  </si>
+  <si>
+    <t>Gao, Antwi-Afari, Huang, Chen &amp; Manzoor - AI in Construction Project Management: systematic review</t>
+  </si>
+  <si>
+    <t>F-15</t>
+  </si>
+  <si>
+    <t>MVCS - Reglamento Nacional de Edificaciones y Norma G.050</t>
+  </si>
+  <si>
+    <t>2006, actualizado</t>
+  </si>
+  <si>
+    <t>Marco técnico obligatorio y seguridad durante la construcción.</t>
+  </si>
+  <si>
+    <t>https://www.gob.pe/institucion/vivienda/informes-publicaciones/2309793-reglamento-nacional-de-edificaciones-rne</t>
+  </si>
+  <si>
+    <t>F-16</t>
+  </si>
+  <si>
+    <t>Congreso - Ley N.º 29783, Ley de Seguridad y Salud en el Trabajo</t>
+  </si>
+  <si>
+    <t>Gestión y registros de seguridad y salud en el trabajo.</t>
+  </si>
+  <si>
+    <t>https://www.gob.pe/institucion/congreso-de-la-republica/normas-legales/462576-29783</t>
+  </si>
+  <si>
+    <t>F-17</t>
+  </si>
+  <si>
+    <t>MTPE - D.S. N.º 011-2019-TR, Reglamento de SST para Construcción</t>
+  </si>
+  <si>
+    <t>Obligaciones sectoriales de SST en obra.</t>
+  </si>
+  <si>
+    <t>https://www.gob.pe/institucion/mtpe/normas-legales/284237-011-2019-tr</t>
+  </si>
+  <si>
+    <t>F-18</t>
+  </si>
+  <si>
+    <t>Congreso - Ley N.º 29733, Ley de Protección de Datos Personales</t>
+  </si>
+  <si>
+    <t>Tratamiento de datos de trabajadores, clientes y proveedores.</t>
+  </si>
+  <si>
+    <t>https://www.gob.pe/institucion/congreso-de-la-republica/normas-legales/243470-29733</t>
+  </si>
+  <si>
+    <t>F-19</t>
+  </si>
+  <si>
+    <t>ANPD - D.S. N.º 016-2024-JUS, Reglamento de la Ley N.º 29733</t>
+  </si>
+  <si>
+    <t>Seguridad, conservación e incidentes de datos personales.</t>
+  </si>
+  <si>
+    <t>https://www.gob.pe/institucion/anpd/normas-legales/6554453-16-2024-jus</t>
   </si>
 </sst>
 </file>
@@ -1268,7 +1349,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:F11"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.796875" defaultRowHeight="13.8"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
@@ -1276,9 +1357,10 @@
     <col min="3" max="3" width="18" customWidth="1"/>
     <col min="4" max="4" width="16" customWidth="1"/>
     <col min="5" max="5" width="52" customWidth="1"/>
+    <col min="6" max="6" width="48.69921875" style="3" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" spans="1:6">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1294,8 +1376,11 @@
       <c r="E1" s="1" t="s">
         <v>64</v>
       </c>
-    </row>
-    <row r="2" spans="1:5" ht="27.6">
+      <c r="F1" s="1" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" ht="27.6">
       <c r="A2" s="3" t="s">
         <v>65</v>
       </c>
@@ -1311,8 +1396,11 @@
       <c r="E2" s="3" t="s">
         <v>69</v>
       </c>
-    </row>
-    <row r="3" spans="1:5" ht="41.4">
+      <c r="F2" s="3" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" ht="41.4">
       <c r="A3" s="3" t="s">
         <v>70</v>
       </c>
@@ -1328,8 +1416,11 @@
       <c r="E3" s="3" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="4" spans="1:5">
+      <c r="F3" s="3" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" ht="27.6">
       <c r="A4" s="3" t="s">
         <v>74</v>
       </c>
@@ -1345,8 +1436,11 @@
       <c r="E4" s="3" t="s">
         <v>76</v>
       </c>
-    </row>
-    <row r="5" spans="1:5" ht="27.6">
+      <c r="F4" s="3" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" ht="27.6">
       <c r="A5" s="3" t="s">
         <v>77</v>
       </c>
@@ -1362,8 +1456,11 @@
       <c r="E5" s="3" t="s">
         <v>79</v>
       </c>
-    </row>
-    <row r="6" spans="1:5" ht="27.6">
+      <c r="F5" s="3" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" ht="27.6">
       <c r="A6" s="3" t="s">
         <v>80</v>
       </c>
@@ -1379,8 +1476,11 @@
       <c r="E6" s="3" t="s">
         <v>82</v>
       </c>
-    </row>
-    <row r="7" spans="1:5" ht="27.6">
+      <c r="F6" s="3" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" ht="27.6">
       <c r="A7" s="3" t="s">
         <v>83</v>
       </c>
@@ -1396,8 +1496,11 @@
       <c r="E7" s="3" t="s">
         <v>76</v>
       </c>
-    </row>
-    <row r="8" spans="1:5" ht="27.6">
+      <c r="F7" s="3" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" ht="27.6">
       <c r="A8" s="3" t="s">
         <v>85</v>
       </c>
@@ -1413,8 +1516,11 @@
       <c r="E8" s="3" t="s">
         <v>87</v>
       </c>
-    </row>
-    <row r="9" spans="1:5" ht="27.6">
+      <c r="F8" s="3" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" ht="27.6">
       <c r="A9" s="3" t="s">
         <v>88</v>
       </c>
@@ -1430,8 +1536,11 @@
       <c r="E9" s="3" t="s">
         <v>91</v>
       </c>
-    </row>
-    <row r="10" spans="1:5" ht="27.6">
+      <c r="F9" s="3" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" ht="27.6">
       <c r="A10" s="3" t="s">
         <v>92</v>
       </c>
@@ -1447,8 +1556,11 @@
       <c r="E10" s="3" t="s">
         <v>96</v>
       </c>
-    </row>
-    <row r="11" spans="1:5" ht="27.6">
+      <c r="F10" s="3" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" ht="27.6">
       <c r="A11" s="3" t="s">
         <v>97</v>
       </c>
@@ -1463,6 +1575,9 @@
       </c>
       <c r="E11" s="3" t="s">
         <v>100</v>
+      </c>
+      <c r="F11" s="3" t="s">
+        <v>227</v>
       </c>
     </row>
   </sheetData>
@@ -1509,7 +1624,7 @@
     </row>
     <row r="2" spans="1:7" ht="27.6">
       <c r="A2" s="3" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="B2" s="3" t="s">
         <v>107</v>
@@ -1521,18 +1636,18 @@
         <v>109</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>220</v>
+        <v>215</v>
       </c>
       <c r="F2" s="3" t="s">
         <v>110</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>213</v>
+        <v>218</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="27.6">
       <c r="A3" s="3" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="B3" s="3" t="s">
         <v>111</v>
@@ -1544,18 +1659,18 @@
         <v>109</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>221</v>
+        <v>216</v>
       </c>
       <c r="F3" s="3" t="s">
         <v>110</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
     </row>
     <row r="4" spans="1:7" ht="27.6">
       <c r="A4" s="3" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="B4" s="3" t="s">
         <v>113</v>
@@ -1573,12 +1688,12 @@
         <v>110</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="27.6">
       <c r="A5" s="3" t="s">
-        <v>218</v>
+        <v>214</v>
       </c>
       <c r="B5" s="3" t="s">
         <v>116</v>
@@ -1590,13 +1705,13 @@
         <v>109</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>222</v>
+        <v>217</v>
       </c>
       <c r="F5" s="3" t="s">
         <v>110</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
     </row>
     <row r="6" spans="1:7">
@@ -1926,7 +2041,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:F15"/>
+  <dimension ref="A1:F20"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.796875" defaultRowHeight="13.8"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
@@ -2185,56 +2300,156 @@
         <v>167</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>172</v>
+        <v>228</v>
       </c>
       <c r="D13" s="3" t="s">
         <v>144</v>
       </c>
       <c r="E13" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="F13" s="3" t="s">
         <v>173</v>
-      </c>
-      <c r="F13" s="3" t="s">
-        <v>174</v>
       </c>
     </row>
     <row r="14" spans="1:6" ht="27.6">
       <c r="A14" s="3" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B14" s="3" t="s">
         <v>124</v>
       </c>
       <c r="C14" s="3" t="s">
+        <v>175</v>
+      </c>
+      <c r="D14" s="3" t="s">
         <v>176</v>
       </c>
-      <c r="D14" s="3" t="s">
+      <c r="E14" s="3" t="s">
         <v>177</v>
       </c>
-      <c r="E14" s="3" t="s">
+      <c r="F14" s="3" t="s">
         <v>178</v>
-      </c>
-      <c r="F14" s="3" t="s">
-        <v>179</v>
       </c>
     </row>
     <row r="15" spans="1:6" ht="27.6">
       <c r="A15" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="B15" s="3" t="s">
         <v>180</v>
       </c>
-      <c r="B15" s="3" t="s">
+      <c r="C15" s="3" t="s">
         <v>181</v>
-      </c>
-      <c r="C15" s="3" t="s">
-        <v>182</v>
       </c>
       <c r="D15" s="3" t="s">
         <v>144</v>
       </c>
       <c r="E15" s="3" t="s">
+        <v>182</v>
+      </c>
+      <c r="F15" s="3" t="s">
         <v>183</v>
       </c>
-      <c r="F15" s="3" t="s">
-        <v>184</v>
+    </row>
+    <row r="16" spans="1:6" ht="27.6">
+      <c r="A16" s="3" t="s">
+        <v>229</v>
+      </c>
+      <c r="B16" s="3">
+        <v>1</v>
+      </c>
+      <c r="C16" s="3" t="s">
+        <v>230</v>
+      </c>
+      <c r="D16" s="3" t="s">
+        <v>231</v>
+      </c>
+      <c r="E16" s="3" t="s">
+        <v>232</v>
+      </c>
+      <c r="F16" s="3" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" ht="27.6">
+      <c r="A17" s="3" t="s">
+        <v>234</v>
+      </c>
+      <c r="B17" s="3">
+        <v>1</v>
+      </c>
+      <c r="C17" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="D17" s="3">
+        <v>2011</v>
+      </c>
+      <c r="E17" s="3" t="s">
+        <v>236</v>
+      </c>
+      <c r="F17" s="3" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" ht="27.6">
+      <c r="A18" s="3" t="s">
+        <v>238</v>
+      </c>
+      <c r="B18" s="3">
+        <v>1</v>
+      </c>
+      <c r="C18" s="3" t="s">
+        <v>239</v>
+      </c>
+      <c r="D18" s="3">
+        <v>2019</v>
+      </c>
+      <c r="E18" s="3" t="s">
+        <v>240</v>
+      </c>
+      <c r="F18" s="3" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" ht="27.6">
+      <c r="A19" s="3" t="s">
+        <v>242</v>
+      </c>
+      <c r="B19" s="3">
+        <v>1</v>
+      </c>
+      <c r="C19" s="3" t="s">
+        <v>243</v>
+      </c>
+      <c r="D19" s="3">
+        <v>2011</v>
+      </c>
+      <c r="E19" s="3" t="s">
+        <v>244</v>
+      </c>
+      <c r="F19" s="3" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" ht="27.6">
+      <c r="A20" s="3" t="s">
+        <v>246</v>
+      </c>
+      <c r="B20" s="3">
+        <v>1</v>
+      </c>
+      <c r="C20" s="3" t="s">
+        <v>247</v>
+      </c>
+      <c r="D20" s="3">
+        <v>2024</v>
+      </c>
+      <c r="E20" s="3" t="s">
+        <v>248</v>
+      </c>
+      <c r="F20" s="3" t="s">
+        <v>249</v>
       </c>
     </row>
   </sheetData>
@@ -2261,19 +2476,19 @@
         <v>0</v>
       </c>
       <c r="B1" s="4" t="s">
+        <v>184</v>
+      </c>
+      <c r="C1" s="4" t="s">
         <v>185</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="D1" s="4" t="s">
         <v>186</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="E1" s="4" t="s">
         <v>187</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="F1" s="4" t="s">
         <v>188</v>
-      </c>
-      <c r="F1" s="4" t="s">
-        <v>189</v>
       </c>
       <c r="G1" s="4" t="s">
         <v>63</v>
@@ -2281,91 +2496,91 @@
     </row>
     <row r="2" spans="1:7" ht="26.4" customHeight="1">
       <c r="A2" s="3" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="B2" s="3" t="s">
         <v>109</v>
       </c>
       <c r="C2" s="3" t="s">
+        <v>190</v>
+      </c>
+      <c r="D2" s="3" t="s">
         <v>191</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="E2" s="3" t="s">
         <v>192</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="F2" s="3" t="s">
         <v>193</v>
       </c>
-      <c r="F2" s="3" t="s">
+      <c r="G2" s="3" t="s">
         <v>194</v>
-      </c>
-      <c r="G2" s="3" t="s">
-        <v>195</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="15" customHeight="1">
       <c r="A3" s="3" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="B3" s="3" t="s">
         <v>109</v>
       </c>
       <c r="C3" s="3" t="s">
+        <v>196</v>
+      </c>
+      <c r="D3" s="3" t="s">
         <v>197</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="E3" s="3" t="s">
         <v>198</v>
       </c>
-      <c r="E3" s="3" t="s">
-        <v>199</v>
-      </c>
       <c r="F3" s="3" t="s">
+        <v>193</v>
+      </c>
+      <c r="G3" s="3" t="s">
         <v>194</v>
-      </c>
-      <c r="G3" s="3" t="s">
-        <v>195</v>
       </c>
     </row>
     <row r="4" spans="1:7" ht="26.4" customHeight="1">
       <c r="A4" s="3" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="B4" s="3" t="s">
         <v>109</v>
       </c>
       <c r="C4" s="3" t="s">
+        <v>200</v>
+      </c>
+      <c r="D4" s="3" t="s">
         <v>201</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="E4" s="3" t="s">
         <v>202</v>
       </c>
-      <c r="E4" s="3" t="s">
-        <v>203</v>
-      </c>
       <c r="F4" s="3" t="s">
+        <v>193</v>
+      </c>
+      <c r="G4" s="3" t="s">
         <v>194</v>
-      </c>
-      <c r="G4" s="3" t="s">
-        <v>195</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="26.4" customHeight="1">
       <c r="A5" s="3" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="B5" s="3" t="s">
         <v>109</v>
       </c>
       <c r="C5" s="3" t="s">
+        <v>204</v>
+      </c>
+      <c r="D5" s="3" t="s">
         <v>205</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="E5" s="3" t="s">
         <v>206</v>
       </c>
-      <c r="E5" s="3" t="s">
-        <v>207</v>
-      </c>
       <c r="F5" s="3" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="G5" s="3" t="s">
         <v>95</v>
@@ -2373,25 +2588,25 @@
     </row>
     <row r="6" spans="1:7" ht="26.4" customHeight="1">
       <c r="A6" s="3" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="B6" s="3" t="s">
         <v>109</v>
       </c>
       <c r="C6" s="3" t="s">
+        <v>208</v>
+      </c>
+      <c r="D6" s="3" t="s">
         <v>209</v>
       </c>
-      <c r="D6" s="3" t="s">
+      <c r="E6" s="3" t="s">
         <v>210</v>
       </c>
-      <c r="E6" s="3" t="s">
-        <v>211</v>
-      </c>
       <c r="F6" s="3" t="s">
+        <v>193</v>
+      </c>
+      <c r="G6" s="3" t="s">
         <v>194</v>
-      </c>
-      <c r="G6" s="3" t="s">
-        <v>195</v>
       </c>
     </row>
   </sheetData>

</xml_diff>